<commit_message>
Add custom HTML frontend and redirect to static index in app.py
</commit_message>
<xml_diff>
--- a/Final_PCW_Filled_With_All_Labors.xlsx
+++ b/Final_PCW_Filled_With_All_Labors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chibi/Desktop/formatting coding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAFEA10-0499-EB41-A38D-9660E4C24B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0A5869-522E-6E44-85E5-8CB8EBA42AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="23240" windowHeight="13880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="660" yWindow="2220" windowWidth="23240" windowHeight="13880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rev 0" sheetId="1" r:id="rId1"/>
@@ -1179,56 +1179,56 @@
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1541,14 +1541,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="137" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="120"/>
       <c r="C1" s="120"/>
       <c r="D1" s="120"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
       <c r="G1" s="120"/>
       <c r="H1" s="120"/>
       <c r="I1" s="130" t="s">
@@ -1558,7 +1558,7 @@
       <c r="K1" s="120"/>
     </row>
     <row r="2" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="119" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="120"/>
@@ -1575,7 +1575,7 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="125" t="s">
+      <c r="A3" s="119" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="120"/>
@@ -1583,8 +1583,8 @@
         <v>5</v>
       </c>
       <c r="D3" s="120"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
       <c r="G3" s="120"/>
       <c r="H3" s="120"/>
       <c r="I3" s="19"/>
@@ -1596,69 +1596,69 @@
       </c>
     </row>
     <row r="4" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="125" t="s">
+      <c r="A4" s="119" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="120"/>
       <c r="C4" s="120"/>
       <c r="D4" s="120"/>
-      <c r="E4" s="127"/>
-      <c r="F4" s="127"/>
+      <c r="E4" s="126"/>
+      <c r="F4" s="126"/>
       <c r="G4" s="120"/>
       <c r="H4" s="120"/>
       <c r="I4" s="19"/>
       <c r="J4" s="8"/>
     </row>
     <row r="5" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="125" t="s">
+      <c r="A5" s="119" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="120"/>
       <c r="C5" s="120"/>
       <c r="D5" s="120"/>
-      <c r="E5" s="127"/>
-      <c r="F5" s="127"/>
+      <c r="E5" s="126"/>
+      <c r="F5" s="126"/>
       <c r="G5" s="120"/>
       <c r="H5" s="120"/>
       <c r="I5" s="19"/>
       <c r="J5" s="8"/>
     </row>
     <row r="6" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="125" t="s">
+      <c r="A6" s="119" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="120"/>
       <c r="C6" s="120"/>
       <c r="D6" s="120"/>
-      <c r="E6" s="127"/>
-      <c r="F6" s="127"/>
+      <c r="E6" s="126"/>
+      <c r="F6" s="126"/>
       <c r="G6" s="120"/>
       <c r="H6" s="120"/>
     </row>
     <row r="7" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="125" t="s">
+      <c r="A7" s="119" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="120"/>
       <c r="C7" s="120"/>
       <c r="D7" s="120"/>
-      <c r="E7" s="127"/>
-      <c r="F7" s="127"/>
+      <c r="E7" s="126"/>
+      <c r="F7" s="126"/>
       <c r="G7" s="120"/>
       <c r="H7" s="120"/>
     </row>
     <row r="8" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="126" t="s">
+      <c r="A8" s="125" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="120"/>
       <c r="C8" s="120"/>
       <c r="D8" s="120"/>
-      <c r="E8" s="127"/>
-      <c r="F8" s="127"/>
+      <c r="E8" s="126"/>
+      <c r="F8" s="126"/>
       <c r="G8" s="120"/>
       <c r="H8" s="120"/>
-      <c r="I8" s="127"/>
+      <c r="I8" s="126"/>
       <c r="J8" s="120"/>
       <c r="K8" s="120"/>
     </row>
@@ -1688,7 +1688,7 @@
       <c r="I9" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="123" t="s">
+      <c r="J9" s="129" t="s">
         <v>20</v>
       </c>
       <c r="K9" s="124"/>
@@ -2551,7 +2551,7 @@
         <f>F38</f>
         <v>0</v>
       </c>
-      <c r="J38" s="135"/>
+      <c r="J38" s="137"/>
       <c r="K38" s="124"/>
       <c r="N38" s="1"/>
       <c r="O38" s="1"/>
@@ -2585,30 +2585,30 @@
       <c r="K39" s="80"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.15">
-      <c r="A40" s="133"/>
+      <c r="A40" s="128"/>
       <c r="B40" s="120"/>
       <c r="C40" s="120"/>
       <c r="D40" s="120"/>
-      <c r="E40" s="127"/>
-      <c r="F40" s="127"/>
+      <c r="E40" s="126"/>
+      <c r="F40" s="126"/>
       <c r="G40" s="120"/>
       <c r="H40" s="120"/>
-      <c r="I40" s="127"/>
+      <c r="I40" s="126"/>
       <c r="J40" s="120"/>
       <c r="K40" s="120"/>
     </row>
     <row r="41" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="126" t="s">
+      <c r="A41" s="125" t="s">
         <v>81</v>
       </c>
       <c r="B41" s="120"/>
       <c r="C41" s="120"/>
       <c r="D41" s="120"/>
-      <c r="E41" s="127"/>
-      <c r="F41" s="127"/>
+      <c r="E41" s="126"/>
+      <c r="F41" s="126"/>
       <c r="G41" s="120"/>
       <c r="H41" s="120"/>
-      <c r="I41" s="127"/>
+      <c r="I41" s="126"/>
       <c r="J41" s="120"/>
       <c r="K41" s="120"/>
     </row>
@@ -2638,7 +2638,7 @@
       <c r="I42" s="84" t="s">
         <v>88</v>
       </c>
-      <c r="J42" s="123" t="s">
+      <c r="J42" s="129" t="s">
         <v>20</v>
       </c>
       <c r="K42" s="124"/>
@@ -3518,7 +3518,7 @@
         <f>D74*G74</f>
         <v>390</v>
       </c>
-      <c r="J74" s="135"/>
+      <c r="J74" s="137"/>
       <c r="K74" s="124"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.15">
@@ -3553,32 +3553,32 @@
       <c r="K75" s="48"/>
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.15">
-      <c r="A76" s="133"/>
+      <c r="A76" s="128"/>
       <c r="B76" s="120"/>
       <c r="C76" s="120"/>
       <c r="D76" s="120"/>
-      <c r="E76" s="127"/>
-      <c r="F76" s="127"/>
+      <c r="E76" s="126"/>
+      <c r="F76" s="126"/>
       <c r="G76" s="120"/>
       <c r="H76" s="120"/>
-      <c r="I76" s="127"/>
+      <c r="I76" s="126"/>
       <c r="J76" s="120"/>
       <c r="K76" s="120"/>
       <c r="N76" s="1"/>
       <c r="S76" s="1"/>
     </row>
     <row r="77" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="126" t="s">
+      <c r="A77" s="125" t="s">
         <v>117</v>
       </c>
       <c r="B77" s="120"/>
       <c r="C77" s="120"/>
       <c r="D77" s="120"/>
-      <c r="E77" s="127"/>
-      <c r="F77" s="127"/>
+      <c r="E77" s="126"/>
+      <c r="F77" s="126"/>
       <c r="G77" s="120"/>
       <c r="H77" s="120"/>
-      <c r="I77" s="127"/>
+      <c r="I77" s="126"/>
       <c r="J77" s="120"/>
       <c r="K77" s="120"/>
     </row>
@@ -3607,7 +3607,7 @@
         <f t="shared" ref="I78:I85" si="7">D78*G78</f>
         <v>110</v>
       </c>
-      <c r="J78" s="119"/>
+      <c r="J78" s="122"/>
       <c r="K78" s="120"/>
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.15">
@@ -3635,7 +3635,7 @@
         <f t="shared" si="7"/>
         <v>220</v>
       </c>
-      <c r="J79" s="119"/>
+      <c r="J79" s="122"/>
       <c r="K79" s="120"/>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.15">
@@ -3663,7 +3663,7 @@
         <f t="shared" si="7"/>
         <v>660</v>
       </c>
-      <c r="J80" s="119"/>
+      <c r="J80" s="122"/>
       <c r="K80" s="120"/>
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.15">
@@ -3691,7 +3691,7 @@
         <f t="shared" si="7"/>
         <v>1540</v>
       </c>
-      <c r="J81" s="119"/>
+      <c r="J81" s="122"/>
       <c r="K81" s="120"/>
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.15">
@@ -3719,7 +3719,7 @@
         <f t="shared" si="7"/>
         <v>220</v>
       </c>
-      <c r="J82" s="119"/>
+      <c r="J82" s="122"/>
       <c r="K82" s="120"/>
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.15">
@@ -3747,7 +3747,7 @@
         <f t="shared" si="7"/>
         <v>110</v>
       </c>
-      <c r="J83" s="119"/>
+      <c r="J83" s="122"/>
       <c r="K83" s="120"/>
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.15">
@@ -3775,7 +3775,7 @@
         <f t="shared" si="7"/>
         <v>110</v>
       </c>
-      <c r="J84" s="119"/>
+      <c r="J84" s="122"/>
       <c r="K84" s="120"/>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.15">
@@ -3803,7 +3803,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J85" s="128"/>
+      <c r="J85" s="133"/>
       <c r="K85" s="124"/>
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.15">
@@ -3836,32 +3836,32 @@
       <c r="K86" s="48"/>
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.15">
-      <c r="A87" s="133"/>
+      <c r="A87" s="128"/>
       <c r="B87" s="120"/>
       <c r="C87" s="120"/>
       <c r="D87" s="120"/>
-      <c r="E87" s="127"/>
-      <c r="F87" s="127"/>
+      <c r="E87" s="126"/>
+      <c r="F87" s="126"/>
       <c r="G87" s="120"/>
       <c r="H87" s="120"/>
-      <c r="I87" s="127"/>
+      <c r="I87" s="126"/>
       <c r="J87" s="120"/>
       <c r="K87" s="120"/>
       <c r="N87" s="1"/>
       <c r="S87" s="1"/>
     </row>
     <row r="88" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="126" t="s">
+      <c r="A88" s="125" t="s">
         <v>126</v>
       </c>
       <c r="B88" s="120"/>
       <c r="C88" s="120"/>
       <c r="D88" s="120"/>
-      <c r="E88" s="127"/>
-      <c r="F88" s="127"/>
+      <c r="E88" s="126"/>
+      <c r="F88" s="126"/>
       <c r="G88" s="120"/>
       <c r="H88" s="120"/>
-      <c r="I88" s="127"/>
+      <c r="I88" s="126"/>
       <c r="J88" s="120"/>
       <c r="K88" s="120"/>
     </row>
@@ -3890,7 +3890,7 @@
         <f t="shared" ref="I89:I94" si="10">D89*G89</f>
         <v>97.5</v>
       </c>
-      <c r="J89" s="119"/>
+      <c r="J89" s="122"/>
       <c r="K89" s="120"/>
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.15">
@@ -3918,7 +3918,7 @@
         <f t="shared" si="10"/>
         <v>195</v>
       </c>
-      <c r="J90" s="119"/>
+      <c r="J90" s="122"/>
       <c r="K90" s="120"/>
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.15">
@@ -3946,7 +3946,7 @@
         <f t="shared" si="10"/>
         <v>107.5</v>
       </c>
-      <c r="J91" s="119"/>
+      <c r="J91" s="122"/>
       <c r="K91" s="120"/>
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.15">
@@ -3974,7 +3974,7 @@
         <f t="shared" si="10"/>
         <v>110</v>
       </c>
-      <c r="J92" s="119"/>
+      <c r="J92" s="122"/>
       <c r="K92" s="120"/>
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.15">
@@ -4002,7 +4002,7 @@
         <f t="shared" si="10"/>
         <v>220</v>
       </c>
-      <c r="J93" s="119"/>
+      <c r="J93" s="122"/>
       <c r="K93" s="120"/>
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.15">
@@ -4030,7 +4030,7 @@
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J94" s="128"/>
+      <c r="J94" s="133"/>
       <c r="K94" s="124"/>
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.15">
@@ -4063,15 +4063,15 @@
       <c r="K95" s="58"/>
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.15">
-      <c r="A96" s="133"/>
+      <c r="A96" s="128"/>
       <c r="B96" s="120"/>
       <c r="C96" s="120"/>
       <c r="D96" s="120"/>
-      <c r="E96" s="127"/>
-      <c r="F96" s="127"/>
+      <c r="E96" s="126"/>
+      <c r="F96" s="126"/>
       <c r="G96" s="120"/>
       <c r="H96" s="120"/>
-      <c r="I96" s="127"/>
+      <c r="I96" s="126"/>
       <c r="J96" s="120"/>
       <c r="K96" s="120"/>
     </row>
@@ -4117,7 +4117,7 @@
         <f t="shared" ref="I98:I104" si="12">D98*G98</f>
         <v>0</v>
       </c>
-      <c r="J98" s="119"/>
+      <c r="J98" s="122"/>
       <c r="K98" s="120"/>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.15">
@@ -4145,7 +4145,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J99" s="119"/>
+      <c r="J99" s="122"/>
       <c r="K99" s="120"/>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.15">
@@ -4173,7 +4173,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J100" s="119"/>
+      <c r="J100" s="122"/>
       <c r="K100" s="120"/>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.15">
@@ -4200,7 +4200,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J101" s="119"/>
+      <c r="J101" s="122"/>
       <c r="K101" s="120"/>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.15">
@@ -4228,7 +4228,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J102" s="119"/>
+      <c r="J102" s="122"/>
       <c r="K102" s="120"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.15">
@@ -4256,7 +4256,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J103" s="119"/>
+      <c r="J103" s="122"/>
       <c r="K103" s="120"/>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.15">
@@ -4282,14 +4282,14 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J104" s="119"/>
+      <c r="J104" s="122"/>
       <c r="K104" s="120"/>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.15">
       <c r="C105" s="11"/>
       <c r="D105" s="70"/>
       <c r="G105" s="23"/>
-      <c r="J105" s="119"/>
+      <c r="J105" s="122"/>
       <c r="K105" s="120"/>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.15">
@@ -4321,7 +4321,7 @@
         <f>B106*G106</f>
         <v>0</v>
       </c>
-      <c r="J106" s="119"/>
+      <c r="J106" s="122"/>
       <c r="K106" s="120"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.15">
@@ -4351,7 +4351,7 @@
         <f t="shared" ref="I107:I112" si="14">F107*G107</f>
         <v>0</v>
       </c>
-      <c r="J107" s="119"/>
+      <c r="J107" s="122"/>
       <c r="K107" s="120"/>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.15">
@@ -4381,7 +4381,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="J108" s="119"/>
+      <c r="J108" s="122"/>
       <c r="K108" s="120"/>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.15">
@@ -4411,7 +4411,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="J109" s="119"/>
+      <c r="J109" s="122"/>
       <c r="K109" s="120"/>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.15">
@@ -4441,7 +4441,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="J110" s="119"/>
+      <c r="J110" s="122"/>
       <c r="K110" s="120"/>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.15">
@@ -4471,7 +4471,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="J111" s="119"/>
+      <c r="J111" s="122"/>
       <c r="K111" s="120"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.15">
@@ -4501,14 +4501,14 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="J112" s="119"/>
+      <c r="J112" s="122"/>
       <c r="K112" s="120"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A113" s="6"/>
       <c r="B113" s="88"/>
       <c r="C113" s="6"/>
-      <c r="J113" s="119"/>
+      <c r="J113" s="122"/>
       <c r="K113" s="120"/>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.15">
@@ -4531,7 +4531,7 @@
         <f>F114*G114</f>
         <v>0</v>
       </c>
-      <c r="J114" s="119"/>
+      <c r="J114" s="122"/>
       <c r="K114" s="120"/>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.15">
@@ -4554,7 +4554,7 @@
         <f>F115*G115</f>
         <v>0</v>
       </c>
-      <c r="J115" s="128"/>
+      <c r="J115" s="133"/>
       <c r="K115" s="124"/>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.15">
@@ -4587,30 +4587,30 @@
       <c r="K116" s="57"/>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A117" s="129"/>
+      <c r="A117" s="135"/>
       <c r="B117" s="120"/>
       <c r="C117" s="120"/>
       <c r="D117" s="120"/>
-      <c r="E117" s="127"/>
-      <c r="F117" s="127"/>
+      <c r="E117" s="126"/>
+      <c r="F117" s="126"/>
       <c r="G117" s="120"/>
       <c r="H117" s="120"/>
-      <c r="I117" s="127"/>
+      <c r="I117" s="126"/>
       <c r="J117" s="120"/>
       <c r="K117" s="120"/>
     </row>
     <row r="118" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="126" t="s">
+      <c r="A118" s="125" t="s">
         <v>158</v>
       </c>
       <c r="B118" s="120"/>
       <c r="C118" s="120"/>
       <c r="D118" s="120"/>
-      <c r="E118" s="127"/>
-      <c r="F118" s="127"/>
+      <c r="E118" s="126"/>
+      <c r="F118" s="126"/>
       <c r="G118" s="120"/>
       <c r="H118" s="120"/>
-      <c r="I118" s="127"/>
+      <c r="I118" s="126"/>
       <c r="J118" s="120"/>
       <c r="K118" s="120"/>
     </row>
@@ -4639,7 +4639,7 @@
         <f>D119*G119</f>
         <v>0</v>
       </c>
-      <c r="J119" s="119"/>
+      <c r="J119" s="122"/>
       <c r="K119" s="120"/>
     </row>
     <row r="120" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4667,7 +4667,7 @@
         <f>D120*G120</f>
         <v>0</v>
       </c>
-      <c r="J120" s="119"/>
+      <c r="J120" s="122"/>
       <c r="K120" s="120"/>
     </row>
     <row r="121" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4695,7 +4695,7 @@
         <f>D121*G121</f>
         <v>0</v>
       </c>
-      <c r="J121" s="119"/>
+      <c r="J121" s="122"/>
       <c r="K121" s="120"/>
     </row>
     <row r="122" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4727,7 +4727,7 @@
         <f>B122*G122</f>
         <v>0</v>
       </c>
-      <c r="J122" s="119"/>
+      <c r="J122" s="122"/>
       <c r="K122" s="120"/>
     </row>
     <row r="123" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4757,7 +4757,7 @@
         <f t="shared" ref="I123:I128" si="16">F123*G123</f>
         <v>0</v>
       </c>
-      <c r="J123" s="119"/>
+      <c r="J123" s="122"/>
       <c r="K123" s="120"/>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.15">
@@ -4787,7 +4787,7 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="J124" s="119"/>
+      <c r="J124" s="122"/>
       <c r="K124" s="120"/>
     </row>
     <row r="125" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4817,7 +4817,7 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="J125" s="119"/>
+      <c r="J125" s="122"/>
       <c r="K125" s="120"/>
     </row>
     <row r="126" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4847,7 +4847,7 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="J126" s="119"/>
+      <c r="J126" s="122"/>
       <c r="K126" s="120"/>
     </row>
     <row r="127" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4877,7 +4877,7 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="J127" s="119"/>
+      <c r="J127" s="122"/>
       <c r="K127" s="120"/>
     </row>
     <row r="128" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4907,7 +4907,7 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="J128" s="128"/>
+      <c r="J128" s="133"/>
       <c r="K128" s="124"/>
     </row>
     <row r="129" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -5186,8 +5186,8 @@
       </c>
       <c r="G146" s="120"/>
       <c r="H146" s="120"/>
-      <c r="I146" s="127"/>
-      <c r="J146" s="122"/>
+      <c r="I146" s="126"/>
+      <c r="J146" s="136"/>
       <c r="K146" s="120"/>
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.15">
@@ -5200,7 +5200,7 @@
       <c r="K147" s="91"/>
     </row>
     <row r="148" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A148" s="136" t="s">
+      <c r="A148" s="123" t="s">
         <v>181</v>
       </c>
       <c r="B148" s="124"/>
@@ -5442,10 +5442,10 @@
         <v>0</v>
       </c>
       <c r="E157" s="132"/>
-      <c r="F157" s="127"/>
+      <c r="F157" s="126"/>
       <c r="G157" s="120"/>
       <c r="H157" s="120"/>
-      <c r="I157" s="127"/>
+      <c r="I157" s="126"/>
       <c r="J157" s="120"/>
       <c r="K157" s="120"/>
     </row>
@@ -5461,11 +5461,11 @@
       <c r="D158" s="71">
         <v>0</v>
       </c>
-      <c r="E158" s="127"/>
-      <c r="F158" s="127"/>
+      <c r="E158" s="126"/>
+      <c r="F158" s="126"/>
       <c r="G158" s="120"/>
       <c r="H158" s="120"/>
-      <c r="I158" s="127"/>
+      <c r="I158" s="126"/>
       <c r="J158" s="120"/>
       <c r="K158" s="120"/>
     </row>
@@ -5481,11 +5481,11 @@
       <c r="D159" s="71">
         <v>0</v>
       </c>
-      <c r="E159" s="127"/>
-      <c r="F159" s="127"/>
+      <c r="E159" s="126"/>
+      <c r="F159" s="126"/>
       <c r="G159" s="120"/>
       <c r="H159" s="120"/>
-      <c r="I159" s="127"/>
+      <c r="I159" s="126"/>
       <c r="J159" s="120"/>
       <c r="K159" s="120"/>
     </row>
@@ -5501,11 +5501,11 @@
       <c r="D160" s="71">
         <v>0</v>
       </c>
-      <c r="E160" s="127"/>
-      <c r="F160" s="127"/>
+      <c r="E160" s="126"/>
+      <c r="F160" s="126"/>
       <c r="G160" s="120"/>
       <c r="H160" s="120"/>
-      <c r="I160" s="127"/>
+      <c r="I160" s="126"/>
       <c r="J160" s="120"/>
       <c r="K160" s="120"/>
     </row>
@@ -5571,20 +5571,85 @@
     </row>
   </sheetData>
   <mergeCells count="127">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="J54:K54"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="J63:K63"/>
-    <mergeCell ref="J124:K124"/>
-    <mergeCell ref="J109:K109"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="J56:K56"/>
-    <mergeCell ref="J90:K90"/>
-    <mergeCell ref="J105:K105"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J126:K126"/>
+    <mergeCell ref="J82:K82"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J146:K146"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J68:K68"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="J111:K111"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J81:K81"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="A87:K87"/>
+    <mergeCell ref="J89:K89"/>
+    <mergeCell ref="J65:K65"/>
+    <mergeCell ref="J74:K74"/>
+    <mergeCell ref="J121:K121"/>
+    <mergeCell ref="J115:K115"/>
+    <mergeCell ref="J122:K122"/>
+    <mergeCell ref="A117:K117"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="J110:K110"/>
+    <mergeCell ref="J64:K64"/>
+    <mergeCell ref="J120:K120"/>
+    <mergeCell ref="J73:K73"/>
+    <mergeCell ref="J57:K57"/>
+    <mergeCell ref="J93:K93"/>
+    <mergeCell ref="J102:K102"/>
+    <mergeCell ref="A88:K88"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J99:K99"/>
+    <mergeCell ref="J61:K61"/>
+    <mergeCell ref="F146:I146"/>
+    <mergeCell ref="J119:K119"/>
+    <mergeCell ref="E157:K160"/>
+    <mergeCell ref="J101:K101"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J103:K103"/>
+    <mergeCell ref="J85:K85"/>
+    <mergeCell ref="J100:K100"/>
+    <mergeCell ref="J94:K94"/>
+    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J114:K114"/>
+    <mergeCell ref="J125:K125"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J108:K108"/>
+    <mergeCell ref="J128:K128"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="J106:K106"/>
+    <mergeCell ref="A96:K96"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="J92:K92"/>
+    <mergeCell ref="J67:K67"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J83:K83"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="C3:H7"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="J62:K62"/>
+    <mergeCell ref="J71:K71"/>
     <mergeCell ref="A148:B148"/>
     <mergeCell ref="A77:K77"/>
     <mergeCell ref="J72:K72"/>
@@ -5609,6 +5674,20 @@
     <mergeCell ref="J79:K79"/>
     <mergeCell ref="J70:K70"/>
     <mergeCell ref="J104:K104"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="J54:K54"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J63:K63"/>
+    <mergeCell ref="J124:K124"/>
+    <mergeCell ref="J109:K109"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="J90:K90"/>
+    <mergeCell ref="J105:K105"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J17:K17"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="J26:K26"/>
     <mergeCell ref="J35:K35"/>
@@ -5619,85 +5698,6 @@
     <mergeCell ref="J91:K91"/>
     <mergeCell ref="J66:K66"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="J106:K106"/>
-    <mergeCell ref="A96:K96"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="A40:K40"/>
-    <mergeCell ref="J92:K92"/>
-    <mergeCell ref="J67:K67"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="J49:K49"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J83:K83"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="F146:I146"/>
-    <mergeCell ref="J119:K119"/>
-    <mergeCell ref="E157:K160"/>
-    <mergeCell ref="J101:K101"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J103:K103"/>
-    <mergeCell ref="J85:K85"/>
-    <mergeCell ref="J100:K100"/>
-    <mergeCell ref="J94:K94"/>
-    <mergeCell ref="A76:K76"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="C3:H7"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="J114:K114"/>
-    <mergeCell ref="J125:K125"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="J51:K51"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="J108:K108"/>
-    <mergeCell ref="J128:K128"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J62:K62"/>
-    <mergeCell ref="J71:K71"/>
-    <mergeCell ref="A117:K117"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="J110:K110"/>
-    <mergeCell ref="J64:K64"/>
-    <mergeCell ref="J120:K120"/>
-    <mergeCell ref="J73:K73"/>
-    <mergeCell ref="J57:K57"/>
-    <mergeCell ref="J93:K93"/>
-    <mergeCell ref="J102:K102"/>
-    <mergeCell ref="A88:K88"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="J99:K99"/>
-    <mergeCell ref="J61:K61"/>
-    <mergeCell ref="J126:K126"/>
-    <mergeCell ref="J82:K82"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J146:K146"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J68:K68"/>
-    <mergeCell ref="J48:K48"/>
-    <mergeCell ref="J111:K111"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J81:K81"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="A87:K87"/>
-    <mergeCell ref="J89:K89"/>
-    <mergeCell ref="J65:K65"/>
-    <mergeCell ref="J74:K74"/>
-    <mergeCell ref="J121:K121"/>
-    <mergeCell ref="J115:K115"/>
-    <mergeCell ref="J122:K122"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="17" scale="51" orientation="portrait" horizontalDpi="4294967292" verticalDpi="1200"/>

</xml_diff>